<commit_message>
Offline mode: suppress component success toast when interceptor just queued the mutation (no duplicate notifications)
</commit_message>
<xml_diff>
--- a/seeders/patients_sample_data.xlsx
+++ b/seeders/patients_sample_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
   <si>
     <t>name</t>
   </si>
@@ -73,55 +73,71 @@
     <t>bloodGroup</t>
   </si>
   <si>
+    <t>Smith Doe</t>
+  </si>
+  <si>
+    <t>sdoe@tiryaq.com</t>
+  </si>
+  <si>
+    <t>1990-03-15</t>
+  </si>
+  <si>
+    <t>+974 5512 3400</t>
+  </si>
+  <si>
+    <t>Qatar Insurance</t>
+  </si>
+  <si>
+    <t>General Surgery</t>
+  </si>
+  <si>
+    <t>Surgery</t>
+  </si>
+  <si>
+    <t>Admitted</t>
+  </si>
+  <si>
+    <t>2025-01-10</t>
+  </si>
+  <si>
+    <t>alkhor</t>
+  </si>
+  <si>
+    <t>Discharged in stable condition with follow-up in 2 weeks</t>
+  </si>
+  <si>
+    <t>Emergency appendectomy January 2024</t>
+  </si>
+  <si>
+    <t>Amoxicillin</t>
+  </si>
+  <si>
+    <t>None currently</t>
+  </si>
+  <si>
+    <t>D104
+D105</t>
+  </si>
+  <si>
+    <t>Surgery Ward</t>
+  </si>
+  <si>
+    <t>O+</t>
+  </si>
+  <si>
     <t>Khalid Ibrahim</t>
   </si>
   <si>
     <t>khalid.ibrahim@email.com</t>
   </si>
   <si>
-    <t>1990-03-15</t>
-  </si>
-  <si>
     <t>male</t>
   </si>
   <si>
     <t>+974 5512 3456</t>
   </si>
   <si>
-    <t>Qatar Insurance</t>
-  </si>
-  <si>
-    <t>General Surgery</t>
-  </si>
-  <si>
-    <t>Surgery</t>
-  </si>
-  <si>
-    <t>Admitted</t>
-  </si>
-  <si>
-    <t>2025-01-10</t>
-  </si>
-  <si>
-    <t>alkhor</t>
-  </si>
-  <si>
-    <t>Discharged in stable condition with follow-up in 2 weeks</t>
-  </si>
-  <si>
-    <t>Emergency appendectomy January 2024</t>
-  </si>
-  <si>
-    <t>Amoxicillin</t>
-  </si>
-  <si>
-    <t>None currently</t>
-  </si>
-  <si>
     <t>D104</t>
-  </si>
-  <si>
-    <t>Surgery Ward</t>
   </si>
   <si>
     <t>AB+</t>
@@ -132,13 +148,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -149,7 +171,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -161,16 +190,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,28 +509,28 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="3" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="3" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="3" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="3" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="3" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="3" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="3" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="3" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="3" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -514,7 +549,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -567,53 +602,110 @@
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="3">
+        <v>28503156000</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="2">
+      <c r="H2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3">
         <v>28503156789</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="1" t="s">
+      <c r="Q3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>36</v>
+      <c r="S3" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(patients): import issues dialog — list bad rows, choose 'Import valid only' or Cancel
</commit_message>
<xml_diff>
--- a/seeders/patients_sample_data.xlsx
+++ b/seeders/patients_sample_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>name</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t>1990-03-15</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>+974 5512 3400</t>
@@ -132,9 +135,6 @@
   </si>
   <si>
     <t>male</t>
-  </si>
-  <si>
-    <t>+974 5512 3456</t>
   </si>
   <si>
     <t>D104</t>
@@ -148,7 +148,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +159,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -190,15 +196,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -512,25 +521,25 @@
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="4" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -592,7 +601,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -602,107 +611,107 @@
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="1"/>
+      <c r="D2" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="3">
-        <v>28503156000</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F2" s="4"/>
       <c r="G2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F3" s="3">
+      <c r="E3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="4">
         <v>28503156789</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>40</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S3" s="1" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
feat(patients): loader during import validation + partial import
</commit_message>
<xml_diff>
--- a/seeders/patients_sample_data.xlsx
+++ b/seeders/patients_sample_data.xlsx
@@ -82,7 +82,7 @@
     <t>1990-03-15</t>
   </si>
   <si>
-    <t/>
+    <t>male</t>
   </si>
   <si>
     <t>+974 5512 3400</t>
@@ -134,7 +134,7 @@
     <t>khalid.ibrahim@email.com</t>
   </si>
   <si>
-    <t>male</t>
+    <t/>
   </si>
   <si>
     <t>D104</t>
@@ -204,11 +204,11 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -611,13 +611,15 @@
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="4"/>
+      <c r="F2" s="3">
+        <v>87878787878</v>
+      </c>
       <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
@@ -669,12 +671,12 @@
         <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>28503156789</v>
       </c>
       <c r="G3" s="1" t="s">

</xml_diff>

<commit_message>
feat(doctors): same import-issues dialog + loader as patients
</commit_message>
<xml_diff>
--- a/seeders/patients_sample_data.xlsx
+++ b/seeders/patients_sample_data.xlsx
@@ -134,7 +134,7 @@
     <t>khalid.ibrahim@email.com</t>
   </si>
   <si>
-    <t/>
+    <t>+97412123232</t>
   </si>
   <si>
     <t>D104</t>
@@ -196,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -206,9 +206,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -521,25 +518,25 @@
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -673,7 +670,7 @@
       <c r="D3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F3" s="3">

</xml_diff>